<commit_message>
added more sample data
</commit_message>
<xml_diff>
--- a/sample_data/complex_sales_workbook.xlsx
+++ b/sample_data/complex_sales_workbook.xlsx
@@ -199,7 +199,7 @@
     <tableColumn id="9" name="NetRevenue"/>
     <tableColumn id="10" name="Status"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
 </table>
 </file>
 
@@ -214,7 +214,7 @@
     <tableColumn id="5" name="Target"/>
     <tableColumn id="6" name="Variance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight11" showRowStripes="1"/>
 </table>
 </file>
 
@@ -230,7 +230,7 @@
     <tableColumn id="6" name="LastCounted"/>
     <tableColumn id="7" name="Warehouse"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -637,18 +637,16 @@
       <c r="H4" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="I4" s="4">
-        <f>F4*G4*(1-H4)</f>
-        <v/>
+      <c r="I4" s="4" t="n">
+        <v>2278.86</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="L4">
-        <f>SUMIF(C4:C15,"North",I4:I15)</f>
-        <v/>
+      <c r="L4" s="4" t="n">
+        <v>11151.16</v>
       </c>
     </row>
     <row r="5">
@@ -684,9 +682,8 @@
       <c r="H5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="4">
-        <f>F5*G5*(1-H5)</f>
-        <v/>
+      <c r="I5" s="4" t="n">
+        <v>2360</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -732,18 +729,16 @@
       <c r="H6" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="I6" s="4">
-        <f>F6*G6*(1-H6)</f>
-        <v/>
+      <c r="I6" s="4" t="n">
+        <v>2686.5</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L6">
-        <f>COUNTIF(J4:J15,"Closed")</f>
-        <v/>
+      <c r="L6" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -779,9 +774,8 @@
       <c r="H7" s="5" t="n">
         <v>0.02</v>
       </c>
-      <c r="I7" s="4">
-        <f>F7*G7*(1-H7)</f>
-        <v/>
+      <c r="I7" s="4" t="n">
+        <v>1175.41</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -827,18 +821,16 @@
       <c r="H8" s="5" t="n">
         <v>0.15</v>
       </c>
-      <c r="I8" s="4">
-        <f>F8*G8*(1-H8)</f>
-        <v/>
+      <c r="I8" s="4" t="n">
+        <v>6526.3</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>Cancelled</t>
         </is>
       </c>
-      <c r="L8">
-        <f>AVERAGE(H4:H15)</f>
-        <v/>
+      <c r="L8" s="5" t="n">
+        <v>0.0592</v>
       </c>
     </row>
     <row r="9" hidden="1">
@@ -874,9 +866,8 @@
       <c r="H9" s="5" t="n">
         <v>0.03</v>
       </c>
-      <c r="I9" s="4">
-        <f>F9*G9*(1-H9)</f>
-        <v/>
+      <c r="I9" s="4" t="n">
+        <v>1731.45</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -917,9 +908,8 @@
       <c r="H10" s="5" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I10" s="4">
-        <f>F10*G10*(1-H10)</f>
-        <v/>
+      <c r="I10" s="4" t="n">
+        <v>2606.32</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -928,7 +918,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Contains blank lines below for parser robustness</t>
+          <t>Row 9 and column K are hidden (parser edge case)</t>
         </is>
       </c>
     </row>
@@ -965,9 +955,8 @@
       <c r="H11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="4">
-        <f>F11*G11*(1-H11)</f>
-        <v/>
+      <c r="I11" s="4" t="n">
+        <v>1791</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1008,9 +997,8 @@
       <c r="H12" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="I12" s="4">
-        <f>F12*G12*(1-H12)</f>
-        <v/>
+      <c r="I12" s="4" t="n">
+        <v>2346</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1051,9 +1039,8 @@
       <c r="H13" s="5" t="n">
         <v>0.12</v>
       </c>
-      <c r="I13" s="4">
-        <f>F13*G13*(1-H13)</f>
-        <v/>
+      <c r="I13" s="4" t="n">
+        <v>5528.16</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1094,9 +1081,8 @@
       <c r="H14" s="5" t="n">
         <v>0.04</v>
       </c>
-      <c r="I14" s="4">
-        <f>F14*G14*(1-H14)</f>
-        <v/>
+      <c r="I14" s="4" t="n">
+        <v>1439.28</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1137,9 +1123,8 @@
       <c r="H15" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="I15" s="4">
-        <f>F15*G15*(1-H15)</f>
-        <v/>
+      <c r="I15" s="4" t="n">
+        <v>3082.75</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1221,24 +1206,20 @@
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4">
-        <f>COUNTIFS(Orders!B:B,"&gt;="&amp;DATE(2025,1,1),Orders!B:B,"&lt;"&amp;DATE(2025,2,1))</f>
-        <v/>
-      </c>
-      <c r="C4" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,1,1),Orders!B:B,"&lt;"&amp;DATE(2025,2,1))</f>
-        <v/>
-      </c>
-      <c r="D4" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,1,1),Orders!B:B,"&lt;"&amp;DATE(2025,2,1),Orders!J:J,"Closed")</f>
-        <v/>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>7325.36</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>4638.86</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>3500</v>
       </c>
-      <c r="F4" s="4">
-        <f>D4-E4</f>
-        <v/>
+      <c r="F4" s="4" t="n">
+        <v>1138.86</v>
       </c>
     </row>
     <row r="5">
@@ -1247,24 +1228,20 @@
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5">
-        <f>COUNTIFS(Orders!B:B,"&gt;="&amp;DATE(2025,2,1),Orders!B:B,"&lt;"&amp;DATE(2025,3,1))</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,2,1),Orders!B:B,"&lt;"&amp;DATE(2025,3,1))</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,2,1),Orders!B:B,"&lt;"&amp;DATE(2025,3,1),Orders!J:J,"Closed")</f>
-        <v/>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>9433.16</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2906.86</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>7000</v>
       </c>
-      <c r="F5" s="4">
-        <f>D5-E5</f>
-        <v/>
+      <c r="F5" s="4" t="n">
+        <v>-4093.14</v>
       </c>
     </row>
     <row r="6">
@@ -1273,24 +1250,20 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6">
-        <f>COUNTIFS(Orders!B:B,"&gt;="&amp;DATE(2025,3,1),Orders!B:B,"&lt;"&amp;DATE(2025,4,1))</f>
-        <v/>
-      </c>
-      <c r="C6" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,3,1),Orders!B:B,"&lt;"&amp;DATE(2025,4,1))</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,3,1),Orders!B:B,"&lt;"&amp;DATE(2025,4,1),Orders!J:J,"Closed")</f>
-        <v/>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>4397.32</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2606.32</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>6500</v>
       </c>
-      <c r="F6" s="4">
-        <f>D6-E6</f>
-        <v/>
+      <c r="F6" s="4" t="n">
+        <v>-3893.68</v>
       </c>
     </row>
     <row r="7">
@@ -1299,24 +1272,20 @@
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7">
-        <f>COUNTIFS(Orders!B:B,"&gt;="&amp;DATE(2025,4,1),Orders!B:B,"&lt;"&amp;DATE(2025,5,1))</f>
-        <v/>
-      </c>
-      <c r="C7" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,4,1),Orders!B:B,"&lt;"&amp;DATE(2025,5,1))</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,4,1),Orders!B:B,"&lt;"&amp;DATE(2025,5,1),Orders!J:J,"Closed")</f>
-        <v/>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>7874.16</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>7874.16</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>8000</v>
       </c>
-      <c r="F7" s="4">
-        <f>D7-E7</f>
-        <v/>
+      <c r="F7" s="4" t="n">
+        <v>-125.84</v>
       </c>
     </row>
     <row r="8">
@@ -1325,24 +1294,20 @@
           <t>May</t>
         </is>
       </c>
-      <c r="B8">
-        <f>COUNTIFS(Orders!B:B,"&gt;="&amp;DATE(2025,5,1),Orders!B:B,"&lt;"&amp;DATE(2025,6,1))</f>
-        <v/>
-      </c>
-      <c r="C8" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,5,1),Orders!B:B,"&lt;"&amp;DATE(2025,6,1))</f>
-        <v/>
-      </c>
-      <c r="D8" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,5,1),Orders!B:B,"&lt;"&amp;DATE(2025,6,1),Orders!J:J,"Closed")</f>
-        <v/>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4522.03</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>3082.75</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>9000</v>
       </c>
-      <c r="F8" s="4">
-        <f>D8-E8</f>
-        <v/>
+      <c r="F8" s="4" t="n">
+        <v>-5917.25</v>
       </c>
     </row>
     <row r="9">
@@ -1351,24 +1316,20 @@
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9">
-        <f>COUNTIFS(Orders!B:B,"&gt;="&amp;DATE(2025,6,1),Orders!B:B,"&lt;"&amp;DATE(2025,7,1))</f>
-        <v/>
-      </c>
-      <c r="C9" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,6,1),Orders!B:B,"&lt;"&amp;DATE(2025,7,1))</f>
-        <v/>
-      </c>
-      <c r="D9" s="4">
-        <f>SUMIFS(Orders!I:I,Orders!B:B,"&gt;="&amp;DATE(2025,6,1),Orders!B:B,"&lt;"&amp;DATE(2025,7,1),Orders!J:J,"Closed")</f>
-        <v/>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="F9" s="4">
-        <f>D9-E9</f>
-        <v/>
+      <c r="F9" s="4" t="n">
+        <v>-10000</v>
       </c>
     </row>
     <row r="11">
@@ -1377,9 +1338,8 @@
           <t>YTD Closed Revenue</t>
         </is>
       </c>
-      <c r="B11" s="4">
-        <f>SUM(D4:D9)</f>
-        <v/>
+      <c r="B11" s="4" t="n">
+        <v>21108.95</v>
       </c>
     </row>
   </sheetData>
@@ -1465,9 +1425,10 @@
       <c r="D2" t="n">
         <v>50</v>
       </c>
-      <c r="E2">
-        <f>IF(C2="","UNKNOWN",IF(C2&lt;=D2,"REORDER","OK"))</f>
-        <v/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>REORDER</t>
+        </is>
       </c>
       <c r="F2" s="3" t="n">
         <v>45778</v>
@@ -1495,9 +1456,10 @@
       <c r="D3" t="n">
         <v>80</v>
       </c>
-      <c r="E3">
-        <f>IF(C3="","UNKNOWN",IF(C3&lt;=D3,"REORDER","OK"))</f>
-        <v/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
       </c>
       <c r="F3" s="3" t="n">
         <v>45787</v>
@@ -1522,11 +1484,11 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4">
-        <f>IF(C4="","UNKNOWN",IF(C4&lt;=D4,"REORDER","OK"))</f>
-        <v/>
-      </c>
-      <c r="F4" s="3" t="n"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1550,9 +1512,10 @@
       <c r="D5" t="n">
         <v>20</v>
       </c>
-      <c r="E5">
-        <f>IF(C5="","UNKNOWN",IF(C5&lt;=D5,"REORDER","OK"))</f>
-        <v/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>REORDER</t>
+        </is>
       </c>
       <c r="F5" s="3" t="n">
         <v>45769</v>
@@ -1580,9 +1543,10 @@
       <c r="D6" t="n">
         <v>25</v>
       </c>
-      <c r="E6">
-        <f>IF(C6="","UNKNOWN",IF(C6&lt;=D6,"REORDER","OK"))</f>
-        <v/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>REORDER</t>
+        </is>
       </c>
       <c r="F6" s="3" t="n">
         <v>45795</v>
@@ -1610,9 +1574,10 @@
       <c r="D7" t="n">
         <v>16</v>
       </c>
-      <c r="E7">
-        <f>IF(C7="","UNKNOWN",IF(C7&lt;=D7,"REORDER","OK"))</f>
-        <v/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>REORDER</t>
+        </is>
       </c>
       <c r="F7" s="3" t="n">
         <v>45700</v>
@@ -1684,7 +1649,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>

</xml_diff>